<commit_message>
feat: support custom employee fields and pending drag flow
</commit_message>
<xml_diff>
--- a/public/employee-template.xlsx
+++ b/public/employee-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="员工名单" sheetId="1" r:id="R50e1cd650e6743f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rcf98b49f5c8a4bab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="员工名单" sheetId="1" r:id="Re3a66f4733ab441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R3284e190546f4bef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -49,7 +49,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -76,6 +76,16 @@
         <x:fgColor rgb="FFEDF2FF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2457E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFD"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="10">
     <x:border/>
@@ -173,7 +183,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="36">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -254,11 +264,64 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EmployeeRoster" displayName="EmployeeRoster" ref="A1:H4" headerRowCount="1">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="员工编号"/>
+    <x:tableColumn id="2" name="姓名"/>
+    <x:tableColumn id="3" name="部门"/>
+    <x:tableColumn id="4" name="岗位"/>
+    <x:tableColumn id="5" name="照片"/>
+    <x:tableColumn id="6" name="工作地点"/>
+    <x:tableColumn id="7" name="司龄"/>
+    <x:tableColumn id="8" name="关键经历"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TemplateGuide" displayName="TemplateGuide" ref="A3:B10" headerRowCount="1">
+  <x:tableColumns count="2">
+    <x:tableColumn id="1" name="字段"/>
+    <x:tableColumn id="2" name="填写要求"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -461,6 +524,9 @@
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -479,6 +545,15 @@
       <x:c r="E1" s="10" t="str">
         <x:v>照片</x:v>
       </x:c>
+      <x:c r="F1" s="45" t="str">
+        <x:v>工作地点</x:v>
+      </x:c>
+      <x:c r="G1" s="45" t="str">
+        <x:v>司龄</x:v>
+      </x:c>
+      <x:c r="H1" s="45" t="str">
+        <x:v>关键经历</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="11" t="str">
@@ -496,6 +571,15 @@
       <x:c r="E2" s="23" t="str">
         <x:v>在此插入照片</x:v>
       </x:c>
+      <x:c r="F2" s="46" t="str">
+        <x:v>上海</x:v>
+      </x:c>
+      <x:c r="G2" s="46" t="str">
+        <x:v>3年</x:v>
+      </x:c>
+      <x:c r="H2" s="46" t="str">
+        <x:v>新产品上市</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="11" t="str">
@@ -513,6 +597,15 @@
       <x:c r="E3" s="23" t="str">
         <x:v>在此插入照片</x:v>
       </x:c>
+      <x:c r="F3" s="46" t="str">
+        <x:v>深圳</x:v>
+      </x:c>
+      <x:c r="G3" s="46" t="str">
+        <x:v>5年</x:v>
+      </x:c>
+      <x:c r="H3" s="46" t="str">
+        <x:v>核心系统重构</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -530,9 +623,21 @@
       <x:c r="E4" s="24" t="str">
         <x:v>在此插入照片</x:v>
       </x:c>
+      <x:c r="F4" s="46" t="str">
+        <x:v>北京</x:v>
+      </x:c>
+      <x:c r="G4" s="46" t="str">
+        <x:v>2年</x:v>
+      </x:c>
+      <x:c r="H4" s="46" t="str">
+        <x:v>新市场开拓</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5208dbdea8a4e68"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
 
@@ -552,6 +657,10 @@
       <x:c r="C1" s="27"/>
       <x:c r="D1" s="27"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+    </x:row>
     <x:row r="3">
       <x:c r="A3" s="30" t="str">
         <x:v>字段</x:v>
@@ -597,7 +706,23 @@
         <x:v>照片</x:v>
       </x:c>
       <x:c r="B8" s="35" t="str">
-        <x:v>选填；在 E 列对应员工行插入图片，建议使用 JPG 或 PNG，一行一张</x:v>
+        <x:v>选填；在“照片”列对应员工行插入 JPG 或 PNG，一行一张</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="48" t="str">
+        <x:v>自定义字段</x:v>
+      </x:c>
+      <x:c r="B9" s="46" t="str">
+        <x:v>可在“照片”列后自由增加列；列名会成为手机端字段名称</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" customHeight="1">
+      <x:c r="A10" s="48" t="str">
+        <x:v>手机展示</x:v>
+      </x:c>
+      <x:c r="B10" s="46" t="str">
+        <x:v>空字段自动隐藏；内容会在手机浏览器中按单列卡片自动换行</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -605,5 +730,8 @@
     <x:mergeCell ref="A1:D1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R201bdd21564b4668"/>
+  </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>